<commit_message>
Fix the first test after styles switch
The file Empty_text_is_written_and_loaded_to_sst test was failing, because
styles part was different.

Mostly make styles part outuput closer to the output of Excel. The original
write most attributes explicitely, new one doesn't write values if they are
implicit. The purpose is to make it easier to compare output with Excel
(e.g. take the original xlsx output, open and save in Excel and then
compare).
</commit_message>
<xml_diff>
--- a/ClosedXML.Tests/Resource/Other/Cells/EmptyText.xlsx
+++ b/ClosedXML.Tests/Resource/Other/Cells/EmptyText.xlsx
@@ -29,61 +29,52 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<x:styleSheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:numFmts count="1">
-    <x:numFmt numFmtId="0" formatCode=""/>
-  </x:numFmts>
-  <x:fonts count="1">
-    <x:font>
-      <x:vertAlign val="baseline"/>
-      <x:sz val="11"/>
-      <x:color rgb="FF000000"/>
-      <x:name val="Calibri"/>
-      <x:family val="2"/>
-    </x:font>
-  </x:fonts>
-  <x:fills count="2">
-    <x:fill>
-      <x:patternFill patternType="none"/>
-    </x:fill>
-    <x:fill>
-      <x:patternFill patternType="gray125"/>
-    </x:fill>
-  </x:fills>
-  <x:borders count="1">
-    <x:border diagonalUp="0" diagonalDown="0">
-      <x:left style="none">
-        <x:color rgb="FF000000"/>
-      </x:left>
-      <x:right style="none">
-        <x:color rgb="FF000000"/>
-      </x:right>
-      <x:top style="none">
-        <x:color rgb="FF000000"/>
-      </x:top>
-      <x:bottom style="none">
-        <x:color rgb="FF000000"/>
-      </x:bottom>
-      <x:diagonal style="none">
-        <x:color rgb="FF000000"/>
-      </x:diagonal>
-    </x:border>
-  </x:borders>
-  <x:cellStyleXfs count="1">
-    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyNumberFormat="1" applyFill="1" applyBorder="0" applyAlignment="1" applyProtection="1">
-      <x:protection locked="1" hidden="0"/>
-    </x:xf>
-  </x:cellStyleXfs>
-  <x:cellXfs count="1">
-    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="0" applyAlignment="1" applyProtection="1">
-      <x:alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="0" indent="0" relativeIndent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <x:protection locked="1" hidden="0"/>
-    </x:xf>
-  </x:cellXfs>
-  <x:cellStyles count="1">
-    <x:cellStyle name="Normal" xfId="0" builtinId="0"/>
-  </x:cellStyles>
-</x:styleSheet>
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <fonts count="1">
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+  </fonts>
+  <fills count="2">
+    <fill>
+      <patternFill patternType="none"/>
+    </fill>
+    <fill>
+      <patternFill patternType="gray125"/>
+    </fill>
+  </fills>
+  <borders count="1">
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+  </borders>
+  <cellStyleXfs count="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+  </cellStyleXfs>
+  <cellXfs count="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+  </cellXfs>
+  <cellStyles count="1">
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+  </cellStyles>
+  <dxfs count="0"/>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
+</styleSheet>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>

</xml_diff>